<commit_message>
credit days,overdue tgt vs achvment comparison drafting done
</commit_message>
<xml_diff>
--- a/Inputs/dealer closing balance shuddo.xlsx
+++ b/Inputs/dealer closing balance shuddo.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21901"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sales_SalesRegister\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CGIT\Desktop\CBL Dealer Report\Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{E79B1C1C-049B-47FA-A4F5-C47F618B5A20}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{190485F6-25C4-41BE-A7F3-5CFBDFE4D049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sales Distributor Ledger1911250" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -4792,7 +4805,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -5338,9 +5351,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -5378,7 +5391,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -5484,7 +5497,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -5626,14 +5639,14 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V1541"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>